<commit_message>
Update Delta Team Sales: Added Hassan (Q3) and Nadeem (Q1-Q3) data
</commit_message>
<xml_diff>
--- a/Delta_Team_Database.xlsx
+++ b/Delta_Team_Database.xlsx
@@ -561,12 +561,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Pending Data</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Pending Data</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3361,6 +3361,966 @@
         <v>136.76</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>hassan</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Hassan</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>631.83</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1177.2</v>
+      </c>
+      <c r="I46" t="n">
+        <v>545.37</v>
+      </c>
+      <c r="J46" t="n">
+        <v>146665.25</v>
+      </c>
+      <c r="K46" t="n">
+        <v>273261.09</v>
+      </c>
+      <c r="L46" t="n">
+        <v>126595.84</v>
+      </c>
+      <c r="M46" t="n">
+        <v>293330.49</v>
+      </c>
+      <c r="N46" t="n">
+        <v>546522.1800000001</v>
+      </c>
+      <c r="O46" t="n">
+        <v>253191.6900000001</v>
+      </c>
+      <c r="P46" t="n">
+        <v>53.67</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>hassan</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Hassan</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>180.9</v>
+      </c>
+      <c r="H47" t="n">
+        <v>227.2</v>
+      </c>
+      <c r="I47" t="n">
+        <v>46.29999999999998</v>
+      </c>
+      <c r="J47" t="n">
+        <v>41991.53</v>
+      </c>
+      <c r="K47" t="n">
+        <v>52739.49</v>
+      </c>
+      <c r="L47" t="n">
+        <v>10747.96</v>
+      </c>
+      <c r="M47" t="n">
+        <v>83983.08</v>
+      </c>
+      <c r="N47" t="n">
+        <v>105478.98</v>
+      </c>
+      <c r="O47" t="n">
+        <v>21495.89999999999</v>
+      </c>
+      <c r="P47" t="n">
+        <v>79.62</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>hassan</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Hassan</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>6737</v>
+      </c>
+      <c r="H48" t="n">
+        <v>4707.02</v>
+      </c>
+      <c r="I48" t="n">
+        <v>-2029.98</v>
+      </c>
+      <c r="J48" t="n">
+        <v>4064396.87</v>
+      </c>
+      <c r="K48" t="n">
+        <v>2839507.14</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-1224889.73</v>
+      </c>
+      <c r="M48" t="n">
+        <v>8128793.75</v>
+      </c>
+      <c r="N48" t="n">
+        <v>5679014.28</v>
+      </c>
+      <c r="O48" t="n">
+        <v>-2449779.47</v>
+      </c>
+      <c r="P48" t="n">
+        <v>143.14</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>hassan</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Hassan</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>656.33</v>
+      </c>
+      <c r="H49" t="n">
+        <v>562</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-94.33000000000004</v>
+      </c>
+      <c r="J49" t="n">
+        <v>439475.69</v>
+      </c>
+      <c r="K49" t="n">
+        <v>376315.2</v>
+      </c>
+      <c r="L49" t="n">
+        <v>-63160.48999999999</v>
+      </c>
+      <c r="M49" t="n">
+        <v>878951.38</v>
+      </c>
+      <c r="N49" t="n">
+        <v>752630.4</v>
+      </c>
+      <c r="O49" t="n">
+        <v>-126320.98</v>
+      </c>
+      <c r="P49" t="n">
+        <v>116.78</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1262.61</v>
+      </c>
+      <c r="H50" t="n">
+        <v>906.5</v>
+      </c>
+      <c r="I50" t="n">
+        <v>-356.1099999999999</v>
+      </c>
+      <c r="J50" t="n">
+        <v>293086.64</v>
+      </c>
+      <c r="K50" t="n">
+        <v>210424.02</v>
+      </c>
+      <c r="L50" t="n">
+        <v>-82662.62000000002</v>
+      </c>
+      <c r="M50" t="n">
+        <v>586173.28</v>
+      </c>
+      <c r="N50" t="n">
+        <v>420848.04</v>
+      </c>
+      <c r="O50" t="n">
+        <v>-165325.24</v>
+      </c>
+      <c r="P50" t="n">
+        <v>139.28</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>1066.83</v>
+      </c>
+      <c r="H51" t="n">
+        <v>205</v>
+      </c>
+      <c r="I51" t="n">
+        <v>-861.8299999999999</v>
+      </c>
+      <c r="J51" t="n">
+        <v>247641.58</v>
+      </c>
+      <c r="K51" t="n">
+        <v>47586.24</v>
+      </c>
+      <c r="L51" t="n">
+        <v>-200055.34</v>
+      </c>
+      <c r="M51" t="n">
+        <v>495283.16</v>
+      </c>
+      <c r="N51" t="n">
+        <v>95172.48</v>
+      </c>
+      <c r="O51" t="n">
+        <v>-400110.68</v>
+      </c>
+      <c r="P51" t="n">
+        <v>520.41</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>3240</v>
+      </c>
+      <c r="H52" t="n">
+        <v>2852</v>
+      </c>
+      <c r="I52" t="n">
+        <v>-388</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1954530</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1720469.01</v>
+      </c>
+      <c r="L52" t="n">
+        <v>-234060.99</v>
+      </c>
+      <c r="M52" t="n">
+        <v>3909060</v>
+      </c>
+      <c r="N52" t="n">
+        <v>3440938.02</v>
+      </c>
+      <c r="O52" t="n">
+        <v>-468121.98</v>
+      </c>
+      <c r="P52" t="n">
+        <v>113.6</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>732.3200000000001</v>
+      </c>
+      <c r="H53" t="n">
+        <v>396</v>
+      </c>
+      <c r="I53" t="n">
+        <v>-336.3200000000001</v>
+      </c>
+      <c r="J53" t="n">
+        <v>490355.28</v>
+      </c>
+      <c r="K53" t="n">
+        <v>265161.6</v>
+      </c>
+      <c r="L53" t="n">
+        <v>-225193.6800000001</v>
+      </c>
+      <c r="M53" t="n">
+        <v>980710.54</v>
+      </c>
+      <c r="N53" t="n">
+        <v>530323.2</v>
+      </c>
+      <c r="O53" t="n">
+        <v>-450387.3400000001</v>
+      </c>
+      <c r="P53" t="n">
+        <v>184.93</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>1613.71</v>
+      </c>
+      <c r="H54" t="n">
+        <v>1870</v>
+      </c>
+      <c r="I54" t="n">
+        <v>256.29</v>
+      </c>
+      <c r="J54" t="n">
+        <v>374586.61</v>
+      </c>
+      <c r="K54" t="n">
+        <v>434079.36</v>
+      </c>
+      <c r="L54" t="n">
+        <v>59492.75</v>
+      </c>
+      <c r="M54" t="n">
+        <v>749173.22</v>
+      </c>
+      <c r="N54" t="n">
+        <v>868158.72</v>
+      </c>
+      <c r="O54" t="n">
+        <v>118985.5</v>
+      </c>
+      <c r="P54" t="n">
+        <v>86.29000000000001</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>670.71</v>
+      </c>
+      <c r="H55" t="n">
+        <v>520.21</v>
+      </c>
+      <c r="I55" t="n">
+        <v>-150.5</v>
+      </c>
+      <c r="J55" t="n">
+        <v>155688.98</v>
+      </c>
+      <c r="K55" t="n">
+        <v>120756.48</v>
+      </c>
+      <c r="L55" t="n">
+        <v>-34932.50000000001</v>
+      </c>
+      <c r="M55" t="n">
+        <v>311377.96</v>
+      </c>
+      <c r="N55" t="n">
+        <v>241512.96</v>
+      </c>
+      <c r="O55" t="n">
+        <v>-69865.00000000003</v>
+      </c>
+      <c r="P55" t="n">
+        <v>128.93</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>140</v>
+      </c>
+      <c r="H56" t="n">
+        <v>480</v>
+      </c>
+      <c r="I56" t="n">
+        <v>340</v>
+      </c>
+      <c r="J56" t="n">
+        <v>84455</v>
+      </c>
+      <c r="K56" t="n">
+        <v>289560</v>
+      </c>
+      <c r="L56" t="n">
+        <v>205105</v>
+      </c>
+      <c r="M56" t="n">
+        <v>168910</v>
+      </c>
+      <c r="N56" t="n">
+        <v>579120</v>
+      </c>
+      <c r="O56" t="n">
+        <v>410210</v>
+      </c>
+      <c r="P56" t="n">
+        <v>29.17</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>1316.65</v>
+      </c>
+      <c r="H57" t="n">
+        <v>623.71</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-692.9400000000001</v>
+      </c>
+      <c r="J57" t="n">
+        <v>881629.16</v>
+      </c>
+      <c r="K57" t="n">
+        <v>417637.56</v>
+      </c>
+      <c r="L57" t="n">
+        <v>-463991.6</v>
+      </c>
+      <c r="M57" t="n">
+        <v>1763258.33</v>
+      </c>
+      <c r="N57" t="n">
+        <v>835275.12</v>
+      </c>
+      <c r="O57" t="n">
+        <v>-927983.2100000001</v>
+      </c>
+      <c r="P57" t="n">
+        <v>211.1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>2239.69</v>
+      </c>
+      <c r="H58" t="n">
+        <v>1605.6</v>
+      </c>
+      <c r="I58" t="n">
+        <v>-634.0900000000001</v>
+      </c>
+      <c r="J58" t="n">
+        <v>519892.88</v>
+      </c>
+      <c r="K58" t="n">
+        <v>372704.73</v>
+      </c>
+      <c r="L58" t="n">
+        <v>-147188.15</v>
+      </c>
+      <c r="M58" t="n">
+        <v>1039785.76</v>
+      </c>
+      <c r="N58" t="n">
+        <v>745409.46</v>
+      </c>
+      <c r="O58" t="n">
+        <v>-294376.3</v>
+      </c>
+      <c r="P58" t="n">
+        <v>139.49</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>365.78</v>
+      </c>
+      <c r="H59" t="n">
+        <v>723.2</v>
+      </c>
+      <c r="I59" t="n">
+        <v>357.4200000000001</v>
+      </c>
+      <c r="J59" t="n">
+        <v>84907.57000000001</v>
+      </c>
+      <c r="K59" t="n">
+        <v>167874.96</v>
+      </c>
+      <c r="L59" t="n">
+        <v>82967.38999999998</v>
+      </c>
+      <c r="M59" t="n">
+        <v>169815.14</v>
+      </c>
+      <c r="N59" t="n">
+        <v>335749.92</v>
+      </c>
+      <c r="O59" t="n">
+        <v>165934.78</v>
+      </c>
+      <c r="P59" t="n">
+        <v>50.58</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>4883</v>
+      </c>
+      <c r="H60" t="n">
+        <v>3493.38</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-1389.62</v>
+      </c>
+      <c r="J60" t="n">
+        <v>2945669.75</v>
+      </c>
+      <c r="K60" t="n">
+        <v>2107382.76</v>
+      </c>
+      <c r="L60" t="n">
+        <v>-838286.9900000002</v>
+      </c>
+      <c r="M60" t="n">
+        <v>5891339.5</v>
+      </c>
+      <c r="N60" t="n">
+        <v>4214765.52</v>
+      </c>
+      <c r="O60" t="n">
+        <v>-1676573.98</v>
+      </c>
+      <c r="P60" t="n">
+        <v>139.78</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>nadeem</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Nadeem</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>1293.56</v>
+      </c>
+      <c r="H61" t="n">
+        <v>1024</v>
+      </c>
+      <c r="I61" t="n">
+        <v>-269.5599999999999</v>
+      </c>
+      <c r="J61" t="n">
+        <v>866164.25</v>
+      </c>
+      <c r="K61" t="n">
+        <v>685670.4</v>
+      </c>
+      <c r="L61" t="n">
+        <v>-180493.85</v>
+      </c>
+      <c r="M61" t="n">
+        <v>1732328.51</v>
+      </c>
+      <c r="N61" t="n">
+        <v>1371340.8</v>
+      </c>
+      <c r="O61" t="n">
+        <v>-360987.71</v>
+      </c>
+      <c r="P61" t="n">
+        <v>126.32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Delta Team Sales: Added Sabah (Q1-Q3) records
</commit_message>
<xml_diff>
--- a/Delta_Team_Database.xlsx
+++ b/Delta_Team_Database.xlsx
@@ -610,7 +610,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Pending Data</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P61"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4321,6 +4321,726 @@
         <v>126.32</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>1003.92</v>
+      </c>
+      <c r="H62" t="n">
+        <v>805</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-198.92</v>
+      </c>
+      <c r="J62" t="n">
+        <v>233036.32</v>
+      </c>
+      <c r="K62" t="n">
+        <v>186863.04</v>
+      </c>
+      <c r="L62" t="n">
+        <v>-46173.28</v>
+      </c>
+      <c r="M62" t="n">
+        <v>466072.63</v>
+      </c>
+      <c r="N62" t="n">
+        <v>373726.08</v>
+      </c>
+      <c r="O62" t="n">
+        <v>-92346.54999999999</v>
+      </c>
+      <c r="P62" t="n">
+        <v>124.71</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>436.35</v>
+      </c>
+      <c r="H63" t="n">
+        <v>166.5</v>
+      </c>
+      <c r="I63" t="n">
+        <v>-269.85</v>
+      </c>
+      <c r="J63" t="n">
+        <v>101289.17</v>
+      </c>
+      <c r="K63" t="n">
+        <v>38649.32</v>
+      </c>
+      <c r="L63" t="n">
+        <v>-62639.85</v>
+      </c>
+      <c r="M63" t="n">
+        <v>202578.34</v>
+      </c>
+      <c r="N63" t="n">
+        <v>77298.64</v>
+      </c>
+      <c r="O63" t="n">
+        <v>-125279.7</v>
+      </c>
+      <c r="P63" t="n">
+        <v>262.07</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>1279.5</v>
+      </c>
+      <c r="H64" t="n">
+        <v>1126</v>
+      </c>
+      <c r="I64" t="n">
+        <v>-153.5</v>
+      </c>
+      <c r="J64" t="n">
+        <v>771858.38</v>
+      </c>
+      <c r="K64" t="n">
+        <v>679259.49</v>
+      </c>
+      <c r="L64" t="n">
+        <v>-92598.89000000001</v>
+      </c>
+      <c r="M64" t="n">
+        <v>1543716.75</v>
+      </c>
+      <c r="N64" t="n">
+        <v>1358518.98</v>
+      </c>
+      <c r="O64" t="n">
+        <v>-185197.77</v>
+      </c>
+      <c r="P64" t="n">
+        <v>113.63</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>526.59</v>
+      </c>
+      <c r="H65" t="n">
+        <v>290.25</v>
+      </c>
+      <c r="I65" t="n">
+        <v>-236.34</v>
+      </c>
+      <c r="J65" t="n">
+        <v>352603.02</v>
+      </c>
+      <c r="K65" t="n">
+        <v>194351.4</v>
+      </c>
+      <c r="L65" t="n">
+        <v>-158251.62</v>
+      </c>
+      <c r="M65" t="n">
+        <v>705206.05</v>
+      </c>
+      <c r="N65" t="n">
+        <v>388702.8</v>
+      </c>
+      <c r="O65" t="n">
+        <v>-316503.2500000001</v>
+      </c>
+      <c r="P65" t="n">
+        <v>181.43</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>743</v>
+      </c>
+      <c r="H66" t="n">
+        <v>1540</v>
+      </c>
+      <c r="I66" t="n">
+        <v>797</v>
+      </c>
+      <c r="J66" t="n">
+        <v>172470.22</v>
+      </c>
+      <c r="K66" t="n">
+        <v>357477.12</v>
+      </c>
+      <c r="L66" t="n">
+        <v>185006.9</v>
+      </c>
+      <c r="M66" t="n">
+        <v>344940.44</v>
+      </c>
+      <c r="N66" t="n">
+        <v>714954.24</v>
+      </c>
+      <c r="O66" t="n">
+        <v>370013.8</v>
+      </c>
+      <c r="P66" t="n">
+        <v>48.25</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>213.45</v>
+      </c>
+      <c r="H67" t="n">
+        <v>274.92</v>
+      </c>
+      <c r="I67" t="n">
+        <v>61.47000000000003</v>
+      </c>
+      <c r="J67" t="n">
+        <v>49548.56</v>
+      </c>
+      <c r="K67" t="n">
+        <v>63816.63</v>
+      </c>
+      <c r="L67" t="n">
+        <v>14268.07</v>
+      </c>
+      <c r="M67" t="n">
+        <v>99097.11</v>
+      </c>
+      <c r="N67" t="n">
+        <v>127633.26</v>
+      </c>
+      <c r="O67" t="n">
+        <v>28536.14999999999</v>
+      </c>
+      <c r="P67" t="n">
+        <v>77.64</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>718.59</v>
+      </c>
+      <c r="H68" t="n">
+        <v>491.25</v>
+      </c>
+      <c r="I68" t="n">
+        <v>-227.34</v>
+      </c>
+      <c r="J68" t="n">
+        <v>433489.42</v>
+      </c>
+      <c r="K68" t="n">
+        <v>296346.57</v>
+      </c>
+      <c r="L68" t="n">
+        <v>-137142.85</v>
+      </c>
+      <c r="M68" t="n">
+        <v>866978.84</v>
+      </c>
+      <c r="N68" t="n">
+        <v>592693.14</v>
+      </c>
+      <c r="O68" t="n">
+        <v>-274285.7</v>
+      </c>
+      <c r="P68" t="n">
+        <v>146.28</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>804.08</v>
+      </c>
+      <c r="H69" t="n">
+        <v>472.06</v>
+      </c>
+      <c r="I69" t="n">
+        <v>-332.02</v>
+      </c>
+      <c r="J69" t="n">
+        <v>538414.85</v>
+      </c>
+      <c r="K69" t="n">
+        <v>316091.38</v>
+      </c>
+      <c r="L69" t="n">
+        <v>-222323.47</v>
+      </c>
+      <c r="M69" t="n">
+        <v>1076829.69</v>
+      </c>
+      <c r="N69" t="n">
+        <v>632182.76</v>
+      </c>
+      <c r="O69" t="n">
+        <v>-444646.9299999999</v>
+      </c>
+      <c r="P69" t="n">
+        <v>170.34</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>1212.68</v>
+      </c>
+      <c r="H70" t="n">
+        <v>1076.4</v>
+      </c>
+      <c r="I70" t="n">
+        <v>-136.28</v>
+      </c>
+      <c r="J70" t="n">
+        <v>281494.76</v>
+      </c>
+      <c r="K70" t="n">
+        <v>249862.59</v>
+      </c>
+      <c r="L70" t="n">
+        <v>-31632.17000000001</v>
+      </c>
+      <c r="M70" t="n">
+        <v>562989.52</v>
+      </c>
+      <c r="N70" t="n">
+        <v>499725.18</v>
+      </c>
+      <c r="O70" t="n">
+        <v>-63264.34000000003</v>
+      </c>
+      <c r="P70" t="n">
+        <v>112.66</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>288.77</v>
+      </c>
+      <c r="H71" t="n">
+        <v>412.8</v>
+      </c>
+      <c r="I71" t="n">
+        <v>124.03</v>
+      </c>
+      <c r="J71" t="n">
+        <v>67033.17999999999</v>
+      </c>
+      <c r="K71" t="n">
+        <v>95822.42999999999</v>
+      </c>
+      <c r="L71" t="n">
+        <v>28789.25</v>
+      </c>
+      <c r="M71" t="n">
+        <v>134066.36</v>
+      </c>
+      <c r="N71" t="n">
+        <v>191644.86</v>
+      </c>
+      <c r="O71" t="n">
+        <v>57578.5</v>
+      </c>
+      <c r="P71" t="n">
+        <v>69.95999999999999</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>1502</v>
+      </c>
+      <c r="H72" t="n">
+        <v>982.65</v>
+      </c>
+      <c r="I72" t="n">
+        <v>-519.35</v>
+      </c>
+      <c r="J72" t="n">
+        <v>906081.5</v>
+      </c>
+      <c r="K72" t="n">
+        <v>592783.53</v>
+      </c>
+      <c r="L72" t="n">
+        <v>-313297.97</v>
+      </c>
+      <c r="M72" t="n">
+        <v>1812163</v>
+      </c>
+      <c r="N72" t="n">
+        <v>1185567.06</v>
+      </c>
+      <c r="O72" t="n">
+        <v>-626595.9399999999</v>
+      </c>
+      <c r="P72" t="n">
+        <v>152.85</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>sabah</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Sabah</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>541.8099999999999</v>
+      </c>
+      <c r="H73" t="n">
+        <v>619</v>
+      </c>
+      <c r="I73" t="n">
+        <v>77.19000000000005</v>
+      </c>
+      <c r="J73" t="n">
+        <v>362790.71</v>
+      </c>
+      <c r="K73" t="n">
+        <v>414482.4</v>
+      </c>
+      <c r="L73" t="n">
+        <v>51691.69</v>
+      </c>
+      <c r="M73" t="n">
+        <v>725581.45</v>
+      </c>
+      <c r="N73" t="n">
+        <v>828964.8</v>
+      </c>
+      <c r="O73" t="n">
+        <v>103383.3500000001</v>
+      </c>
+      <c r="P73" t="n">
+        <v>87.53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Delta Team Sales: Added Tawfik (Q1-Q3) records
</commit_message>
<xml_diff>
--- a/Delta_Team_Database.xlsx
+++ b/Delta_Team_Database.xlsx
@@ -632,7 +632,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pending Data</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P73"/>
+  <dimension ref="A1:P85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5041,6 +5041,726 @@
         <v>87.53</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>877.77</v>
+      </c>
+      <c r="H74" t="n">
+        <v>602</v>
+      </c>
+      <c r="I74" t="n">
+        <v>-275.77</v>
+      </c>
+      <c r="J74" t="n">
+        <v>203755.28</v>
+      </c>
+      <c r="K74" t="n">
+        <v>139741.05</v>
+      </c>
+      <c r="L74" t="n">
+        <v>-64014.23000000001</v>
+      </c>
+      <c r="M74" t="n">
+        <v>407510.55</v>
+      </c>
+      <c r="N74" t="n">
+        <v>279482.1</v>
+      </c>
+      <c r="O74" t="n">
+        <v>-128028.45</v>
+      </c>
+      <c r="P74" t="n">
+        <v>145.81</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>631.8099999999999</v>
+      </c>
+      <c r="H75" t="n">
+        <v>227.5</v>
+      </c>
+      <c r="I75" t="n">
+        <v>-404.3099999999999</v>
+      </c>
+      <c r="J75" t="n">
+        <v>146660.21</v>
+      </c>
+      <c r="K75" t="n">
+        <v>52809.12</v>
+      </c>
+      <c r="L75" t="n">
+        <v>-93851.09</v>
+      </c>
+      <c r="M75" t="n">
+        <v>293320.42</v>
+      </c>
+      <c r="N75" t="n">
+        <v>105618.24</v>
+      </c>
+      <c r="O75" t="n">
+        <v>-187702.18</v>
+      </c>
+      <c r="P75" t="n">
+        <v>277.72</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>3010.5</v>
+      </c>
+      <c r="H76" t="n">
+        <v>2646</v>
+      </c>
+      <c r="I76" t="n">
+        <v>-364.5</v>
+      </c>
+      <c r="J76" t="n">
+        <v>1816084.12</v>
+      </c>
+      <c r="K76" t="n">
+        <v>1596199.5</v>
+      </c>
+      <c r="L76" t="n">
+        <v>-219884.6200000001</v>
+      </c>
+      <c r="M76" t="n">
+        <v>3632168.25</v>
+      </c>
+      <c r="N76" t="n">
+        <v>3192399</v>
+      </c>
+      <c r="O76" t="n">
+        <v>-439769.25</v>
+      </c>
+      <c r="P76" t="n">
+        <v>113.78</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>653.63</v>
+      </c>
+      <c r="H77" t="n">
+        <v>386.25</v>
+      </c>
+      <c r="I77" t="n">
+        <v>-267.38</v>
+      </c>
+      <c r="J77" t="n">
+        <v>437667.13</v>
+      </c>
+      <c r="K77" t="n">
+        <v>258633</v>
+      </c>
+      <c r="L77" t="n">
+        <v>-179034.13</v>
+      </c>
+      <c r="M77" t="n">
+        <v>875334.26</v>
+      </c>
+      <c r="N77" t="n">
+        <v>517266</v>
+      </c>
+      <c r="O77" t="n">
+        <v>-358068.26</v>
+      </c>
+      <c r="P77" t="n">
+        <v>169.22</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>699.99</v>
+      </c>
+      <c r="H78" t="n">
+        <v>1295</v>
+      </c>
+      <c r="I78" t="n">
+        <v>595.01</v>
+      </c>
+      <c r="J78" t="n">
+        <v>162487.3</v>
+      </c>
+      <c r="K78" t="n">
+        <v>300605.76</v>
+      </c>
+      <c r="L78" t="n">
+        <v>138118.46</v>
+      </c>
+      <c r="M78" t="n">
+        <v>324974.6</v>
+      </c>
+      <c r="N78" t="n">
+        <v>601211.52</v>
+      </c>
+      <c r="O78" t="n">
+        <v>276236.92</v>
+      </c>
+      <c r="P78" t="n">
+        <v>54.05</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>477.78</v>
+      </c>
+      <c r="H79" t="n">
+        <v>312.84</v>
+      </c>
+      <c r="I79" t="n">
+        <v>-164.94</v>
+      </c>
+      <c r="J79" t="n">
+        <v>110907.79</v>
+      </c>
+      <c r="K79" t="n">
+        <v>72618.92999999999</v>
+      </c>
+      <c r="L79" t="n">
+        <v>-38288.86</v>
+      </c>
+      <c r="M79" t="n">
+        <v>221815.58</v>
+      </c>
+      <c r="N79" t="n">
+        <v>145237.86</v>
+      </c>
+      <c r="O79" t="n">
+        <v>-76577.72</v>
+      </c>
+      <c r="P79" t="n">
+        <v>152.73</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>615.41</v>
+      </c>
+      <c r="H80" t="n">
+        <v>498.75</v>
+      </c>
+      <c r="I80" t="n">
+        <v>-116.66</v>
+      </c>
+      <c r="J80" t="n">
+        <v>371246.08</v>
+      </c>
+      <c r="K80" t="n">
+        <v>300870.93</v>
+      </c>
+      <c r="L80" t="n">
+        <v>-70375.15000000002</v>
+      </c>
+      <c r="M80" t="n">
+        <v>742492.17</v>
+      </c>
+      <c r="N80" t="n">
+        <v>601741.86</v>
+      </c>
+      <c r="O80" t="n">
+        <v>-140750.3100000001</v>
+      </c>
+      <c r="P80" t="n">
+        <v>123.39</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>758.9400000000001</v>
+      </c>
+      <c r="H81" t="n">
+        <v>587.4</v>
+      </c>
+      <c r="I81" t="n">
+        <v>-171.5400000000001</v>
+      </c>
+      <c r="J81" t="n">
+        <v>508194.59</v>
+      </c>
+      <c r="K81" t="n">
+        <v>393323.04</v>
+      </c>
+      <c r="L81" t="n">
+        <v>-114871.55</v>
+      </c>
+      <c r="M81" t="n">
+        <v>1016389.19</v>
+      </c>
+      <c r="N81" t="n">
+        <v>786646.08</v>
+      </c>
+      <c r="O81" t="n">
+        <v>-229743.11</v>
+      </c>
+      <c r="P81" t="n">
+        <v>129.21</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>1214.43</v>
+      </c>
+      <c r="H82" t="n">
+        <v>928.8</v>
+      </c>
+      <c r="I82" t="n">
+        <v>-285.6300000000001</v>
+      </c>
+      <c r="J82" t="n">
+        <v>281903.62</v>
+      </c>
+      <c r="K82" t="n">
+        <v>215600.49</v>
+      </c>
+      <c r="L82" t="n">
+        <v>-66303.13</v>
+      </c>
+      <c r="M82" t="n">
+        <v>563807.25</v>
+      </c>
+      <c r="N82" t="n">
+        <v>431200.98</v>
+      </c>
+      <c r="O82" t="n">
+        <v>-132606.27</v>
+      </c>
+      <c r="P82" t="n">
+        <v>130.75</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>313.33</v>
+      </c>
+      <c r="H83" t="n">
+        <v>475.2</v>
+      </c>
+      <c r="I83" t="n">
+        <v>161.87</v>
+      </c>
+      <c r="J83" t="n">
+        <v>72731.78</v>
+      </c>
+      <c r="K83" t="n">
+        <v>110307.24</v>
+      </c>
+      <c r="L83" t="n">
+        <v>37575.46000000001</v>
+      </c>
+      <c r="M83" t="n">
+        <v>145463.57</v>
+      </c>
+      <c r="N83" t="n">
+        <v>220614.48</v>
+      </c>
+      <c r="O83" t="n">
+        <v>75150.91</v>
+      </c>
+      <c r="P83" t="n">
+        <v>65.94</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>3558</v>
+      </c>
+      <c r="H84" t="n">
+        <v>2525.44</v>
+      </c>
+      <c r="I84" t="n">
+        <v>-1032.56</v>
+      </c>
+      <c r="J84" t="n">
+        <v>2146363.5</v>
+      </c>
+      <c r="K84" t="n">
+        <v>1523473.98</v>
+      </c>
+      <c r="L84" t="n">
+        <v>-622889.52</v>
+      </c>
+      <c r="M84" t="n">
+        <v>4292727</v>
+      </c>
+      <c r="N84" t="n">
+        <v>3046947.96</v>
+      </c>
+      <c r="O84" t="n">
+        <v>-1245779.04</v>
+      </c>
+      <c r="P84" t="n">
+        <v>140.89</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>tawfik</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Tawfik</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>667.55</v>
+      </c>
+      <c r="H85" t="n">
+        <v>671</v>
+      </c>
+      <c r="I85" t="n">
+        <v>3.450000000000045</v>
+      </c>
+      <c r="J85" t="n">
+        <v>446994.4</v>
+      </c>
+      <c r="K85" t="n">
+        <v>449301.6</v>
+      </c>
+      <c r="L85" t="n">
+        <v>2307.199999999953</v>
+      </c>
+      <c r="M85" t="n">
+        <v>893988.79</v>
+      </c>
+      <c r="N85" t="n">
+        <v>898603.2</v>
+      </c>
+      <c r="O85" t="n">
+        <v>4614.409999999916</v>
+      </c>
+      <c r="P85" t="n">
+        <v>99.48999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Delta Team sales with Wedad Q1-Q3 files (All 9 reps now active)
</commit_message>
<xml_diff>
--- a/Delta_Team_Database.xlsx
+++ b/Delta_Team_Database.xlsx
@@ -435,7 +435,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -654,7 +654,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Pending Data</t>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P85"/>
+  <dimension ref="A1:P97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5761,6 +5761,726 @@
         <v>99.48999999999999</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>572.36</v>
+      </c>
+      <c r="H86" t="n">
+        <v>918.75</v>
+      </c>
+      <c r="I86" t="n">
+        <v>346.39</v>
+      </c>
+      <c r="J86" t="n">
+        <v>132859.33</v>
+      </c>
+      <c r="K86" t="n">
+        <v>213267.6</v>
+      </c>
+      <c r="L86" t="n">
+        <v>80408.27000000002</v>
+      </c>
+      <c r="M86" t="n">
+        <v>265718.66</v>
+      </c>
+      <c r="N86" t="n">
+        <v>426535.2</v>
+      </c>
+      <c r="O86" t="n">
+        <v>160816.54</v>
+      </c>
+      <c r="P86" t="n">
+        <v>62.3</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>539.33</v>
+      </c>
+      <c r="H87" t="n">
+        <v>247.5</v>
+      </c>
+      <c r="I87" t="n">
+        <v>-291.83</v>
+      </c>
+      <c r="J87" t="n">
+        <v>125194.17</v>
+      </c>
+      <c r="K87" t="n">
+        <v>57451.68</v>
+      </c>
+      <c r="L87" t="n">
+        <v>-67742.48999999999</v>
+      </c>
+      <c r="M87" t="n">
+        <v>250388.35</v>
+      </c>
+      <c r="N87" t="n">
+        <v>114903.36</v>
+      </c>
+      <c r="O87" t="n">
+        <v>-135484.99</v>
+      </c>
+      <c r="P87" t="n">
+        <v>217.91</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>1701.5</v>
+      </c>
+      <c r="H88" t="n">
+        <v>1498</v>
+      </c>
+      <c r="I88" t="n">
+        <v>-203.5</v>
+      </c>
+      <c r="J88" t="n">
+        <v>1026429.88</v>
+      </c>
+      <c r="K88" t="n">
+        <v>903668.49</v>
+      </c>
+      <c r="L88" t="n">
+        <v>-122761.39</v>
+      </c>
+      <c r="M88" t="n">
+        <v>2052859.75</v>
+      </c>
+      <c r="N88" t="n">
+        <v>1807336.98</v>
+      </c>
+      <c r="O88" t="n">
+        <v>-245522.77</v>
+      </c>
+      <c r="P88" t="n">
+        <v>113.58</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="H89" t="n">
+        <v>433.5</v>
+      </c>
+      <c r="I89" t="n">
+        <v>360.6</v>
+      </c>
+      <c r="J89" t="n">
+        <v>48811.96</v>
+      </c>
+      <c r="K89" t="n">
+        <v>290271.6</v>
+      </c>
+      <c r="L89" t="n">
+        <v>241459.64</v>
+      </c>
+      <c r="M89" t="n">
+        <v>97623.92999999999</v>
+      </c>
+      <c r="N89" t="n">
+        <v>580543.2</v>
+      </c>
+      <c r="O89" t="n">
+        <v>482919.27</v>
+      </c>
+      <c r="P89" t="n">
+        <v>16.82</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>506.41</v>
+      </c>
+      <c r="H90" t="n">
+        <v>1262.5</v>
+      </c>
+      <c r="I90" t="n">
+        <v>756.0899999999999</v>
+      </c>
+      <c r="J90" t="n">
+        <v>117551.3</v>
+      </c>
+      <c r="K90" t="n">
+        <v>293061.6</v>
+      </c>
+      <c r="L90" t="n">
+        <v>175510.3</v>
+      </c>
+      <c r="M90" t="n">
+        <v>235102.59</v>
+      </c>
+      <c r="N90" t="n">
+        <v>586123.2</v>
+      </c>
+      <c r="O90" t="n">
+        <v>351020.61</v>
+      </c>
+      <c r="P90" t="n">
+        <v>40.11</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>451.69</v>
+      </c>
+      <c r="H91" t="n">
+        <v>437.26</v>
+      </c>
+      <c r="I91" t="n">
+        <v>-14.43000000000001</v>
+      </c>
+      <c r="J91" t="n">
+        <v>104851.33</v>
+      </c>
+      <c r="K91" t="n">
+        <v>101501.46</v>
+      </c>
+      <c r="L91" t="n">
+        <v>-3349.869999999995</v>
+      </c>
+      <c r="M91" t="n">
+        <v>209702.67</v>
+      </c>
+      <c r="N91" t="n">
+        <v>203002.92</v>
+      </c>
+      <c r="O91" t="n">
+        <v>-6699.75</v>
+      </c>
+      <c r="P91" t="n">
+        <v>103.3</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>490</v>
+      </c>
+      <c r="H92" t="n">
+        <v>287.5</v>
+      </c>
+      <c r="I92" t="n">
+        <v>-202.5</v>
+      </c>
+      <c r="J92" t="n">
+        <v>295592.5</v>
+      </c>
+      <c r="K92" t="n">
+        <v>173434.38</v>
+      </c>
+      <c r="L92" t="n">
+        <v>-122158.12</v>
+      </c>
+      <c r="M92" t="n">
+        <v>591185</v>
+      </c>
+      <c r="N92" t="n">
+        <v>346868.76</v>
+      </c>
+      <c r="O92" t="n">
+        <v>-244316.24</v>
+      </c>
+      <c r="P92" t="n">
+        <v>170.43</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>634.1900000000001</v>
+      </c>
+      <c r="H93" t="n">
+        <v>582.0599999999999</v>
+      </c>
+      <c r="I93" t="n">
+        <v>-52.13000000000011</v>
+      </c>
+      <c r="J93" t="n">
+        <v>424649.77</v>
+      </c>
+      <c r="K93" t="n">
+        <v>389747.37</v>
+      </c>
+      <c r="L93" t="n">
+        <v>-34902.40000000002</v>
+      </c>
+      <c r="M93" t="n">
+        <v>849299.55</v>
+      </c>
+      <c r="N93" t="n">
+        <v>779494.74</v>
+      </c>
+      <c r="O93" t="n">
+        <v>-69804.81000000006</v>
+      </c>
+      <c r="P93" t="n">
+        <v>108.96</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284.02</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Humaxin Mix 70/30</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>718.79</v>
+      </c>
+      <c r="H94" t="n">
+        <v>817.2</v>
+      </c>
+      <c r="I94" t="n">
+        <v>98.41000000000008</v>
+      </c>
+      <c r="J94" t="n">
+        <v>166851.68</v>
+      </c>
+      <c r="K94" t="n">
+        <v>189695.01</v>
+      </c>
+      <c r="L94" t="n">
+        <v>22843.33000000002</v>
+      </c>
+      <c r="M94" t="n">
+        <v>333703.36</v>
+      </c>
+      <c r="N94" t="n">
+        <v>379390.02</v>
+      </c>
+      <c r="O94" t="n">
+        <v>45686.66000000003</v>
+      </c>
+      <c r="P94" t="n">
+        <v>87.95999999999999</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFP-CD-0284</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Humaxin Rapid</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>210.79</v>
+      </c>
+      <c r="H95" t="n">
+        <v>612</v>
+      </c>
+      <c r="I95" t="n">
+        <v>401.21</v>
+      </c>
+      <c r="J95" t="n">
+        <v>48931.89</v>
+      </c>
+      <c r="K95" t="n">
+        <v>142062.33</v>
+      </c>
+      <c r="L95" t="n">
+        <v>93130.43999999999</v>
+      </c>
+      <c r="M95" t="n">
+        <v>97863.77</v>
+      </c>
+      <c r="N95" t="n">
+        <v>284124.66</v>
+      </c>
+      <c r="O95" t="n">
+        <v>186260.89</v>
+      </c>
+      <c r="P95" t="n">
+        <v>34.44</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>1251</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.05</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Glargivin UPA</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>1577</v>
+      </c>
+      <c r="H96" t="n">
+        <v>1031.72</v>
+      </c>
+      <c r="I96" t="n">
+        <v>-545.28</v>
+      </c>
+      <c r="J96" t="n">
+        <v>951325.25</v>
+      </c>
+      <c r="K96" t="n">
+        <v>622383.24</v>
+      </c>
+      <c r="L96" t="n">
+        <v>-328942.01</v>
+      </c>
+      <c r="M96" t="n">
+        <v>1902650.5</v>
+      </c>
+      <c r="N96" t="n">
+        <v>1244766.48</v>
+      </c>
+      <c r="O96" t="n">
+        <v>-657884.02</v>
+      </c>
+      <c r="P96" t="n">
+        <v>152.85</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>wedad</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Wedad</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>OFP-CD-0326.03</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Glargivin 100IU</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>625.85</v>
+      </c>
+      <c r="H97" t="n">
+        <v>486</v>
+      </c>
+      <c r="I97" t="n">
+        <v>-139.85</v>
+      </c>
+      <c r="J97" t="n">
+        <v>419068.89</v>
+      </c>
+      <c r="K97" t="n">
+        <v>325425.6</v>
+      </c>
+      <c r="L97" t="n">
+        <v>-93643.29000000004</v>
+      </c>
+      <c r="M97" t="n">
+        <v>838137.78</v>
+      </c>
+      <c r="N97" t="n">
+        <v>650851.2</v>
+      </c>
+      <c r="O97" t="n">
+        <v>-187286.5800000001</v>
+      </c>
+      <c r="P97" t="n">
+        <v>128.78</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>